<commit_message>
actualizacion mas reciente de proeycto
</commit_message>
<xml_diff>
--- a/Horas_Beca.xlsx
+++ b/Horas_Beca.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\James\Desktop\BecaGo\django-crud-auth TERMINADO CON ESTILOS\ACTUALIZADO\Prototipo Programado\django-crud-auth\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\James\Desktop\XITU\django-crud-auth\django-crud-auth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FF9418-D911-432E-957A-3C8A6C61AEFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C49BF1-9840-4E74-8203-6A1EA7E0F18C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Usuario</t>
   </si>
@@ -58,6 +58,21 @@
   </si>
   <si>
     <t>zam25966</t>
+  </si>
+  <si>
+    <t>alt22568</t>
+  </si>
+  <si>
+    <t>bat25674</t>
+  </si>
+  <si>
+    <t>xit25783</t>
+  </si>
+  <si>
+    <t>che25896</t>
+  </si>
+  <si>
+    <t>men25255</t>
   </si>
 </sst>
 </file>
@@ -375,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -463,6 +478,46 @@
         <v>40</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>